<commit_message>
update several example scripts to reflect the ZCU111 RFdc ADC output current changes.
</commit_message>
<xml_diff>
--- a/examples/zcu111/real_send_real_recv/images/figures.xlsx
+++ b/examples/zcu111/real_send_real_recv/images/figures.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\document\e-trees\Q-LEAP\e7awg_porting\e7awg_sw_simple_multi\examples\zcu111\real_send_real_recv\images\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9442F94B-A7EC-446E-8B6C-E658D89CA164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{277FD6F3-AF27-40DF-91D6-A39CD6F48CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="20925" tabRatio="674" xr2:uid="{8801B8C6-3D98-4B0B-A0B5-1E828D53B5C6}"/>
   </bookViews>
@@ -101,22 +101,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>635054</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>189379</xdr:rowOff>
+      <xdr:colOff>647700</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>190499</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>397824</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>198916</xdr:rowOff>
+      <xdr:colOff>442533</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>36624</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="図 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72424D9A-113B-B47E-F2A0-96708D76EBE7}"/>
+        <xdr:cNvPr id="4" name="図 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CF6CCEDC-7BF4-8712-3D40-18CEC0F344CA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -125,7 +125,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -138,8 +138,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1318613" y="6072467"/>
-          <a:ext cx="7281917" cy="5421978"/>
+          <a:off x="1331259" y="6308911"/>
+          <a:ext cx="7313980" cy="5493889"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -284,13 +284,13 @@
       <xdr:col>5</xdr:col>
       <xdr:colOff>50135</xdr:colOff>
       <xdr:row>48</xdr:row>
-      <xdr:rowOff>59997</xdr:rowOff>
+      <xdr:rowOff>149645</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>425824</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>211530</xdr:rowOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>65855</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -305,7 +305,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3467929" y="11355526"/>
+          <a:off x="3467929" y="11445174"/>
           <a:ext cx="3109924" cy="386857"/>
         </a:xfrm>
         <a:prstGeom prst="rect">

</xml_diff>